<commit_message>
adjustment kolom and number format for qty
</commit_message>
<xml_diff>
--- a/public/assets/example/contoh-import-penerimaan-gudang-input.xlsx
+++ b/public/assets/example/contoh-import-penerimaan-gudang-input.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASBAZAR\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\nds_wip\public\assets\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53774EB2-4C8C-421C-A3E6-A17ED50BF2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D96286-228A-4C64-8541-7D9937CC5AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>buyer</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>A.1.1</t>
+  </si>
+  <si>
+    <t>FABRIC</t>
   </si>
 </sst>
 </file>
@@ -91,7 +94,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -171,7 +174,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
@@ -685,8 +688,8 @@
     <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="7.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="12.5703125" customWidth="1"/>
     <col min="10" max="10" width="28.140625" customWidth="1"/>
@@ -695,31 +698,31 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>1</v>
@@ -728,30 +731,32 @@
       <c r="M1" s="5"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="3">
-        <v>1</v>
+      <c r="A2" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="4">
+      <c r="F2" s="4">
         <v>1</v>
       </c>
-      <c r="F2" s="4">
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4">
         <v>25</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>2</v>

</xml_diff>